<commit_message>
#1 MOdule Step file added
</commit_message>
<xml_diff>
--- a/Design-Files/ASCII-v1.1/BOM/Client-BOM-ASCII-v1.1.xlsx
+++ b/Design-Files/ASCII-v1.1/BOM/Client-BOM-ASCII-v1.1.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="193">
   <si>
     <t>#</t>
   </si>
@@ -586,6 +586,18 @@
   </si>
   <si>
     <t>ROHM Semicon</t>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>DEV-15583</t>
+  </si>
+  <si>
+    <t>SparkFun Electronics</t>
+  </si>
+  <si>
+    <t>RT1062 Teensy 4.0 i.MX ARM® Cortex®-M7 MPU Embedded Evaluation Board</t>
   </si>
 </sst>
 </file>
@@ -1078,7 +1090,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1174,7 +1186,7 @@
     <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B36" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B37" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -2226,6 +2238,37 @@
         <v>1</v>
       </c>
       <c r="K36" s="9"/>
+    </row>
+    <row r="37" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="11">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="G37" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="H37" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="I37" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="J37" s="9">
+        <v>1</v>
+      </c>
+      <c r="K37" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>